<commit_message>
docs(v3.1.21): finalize release metadata and distribution checksums
</commit_message>
<xml_diff>
--- a/wbs/FDS_v3.1.21_WBS_and_Gantt_v1.0.xlsx
+++ b/wbs/FDS_v3.1.21_WBS_and_Gantt_v1.0.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R474dd0636d594c11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="R3ccb21fef7674a45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R4b6fdec12f0b4bbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R39fbcf6eabbd4924"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R8216eeee5ad74577"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="R5bb63d6f8f624e97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R7f229f3e37e84c35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R45eaa95bd7b34e97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Raa470296588e4f92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="R68e50c9898c44576"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4c4904ef6c724dd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS" sheetId="2" r:id="Rdba9609e192e4f12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 Gantt" sheetId="3" r:id="R9f8c687080eb4e9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 Gantt" sheetId="4" r:id="R73e6ec60812a48ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones &amp; Decisions" sheetId="5" r:id="R0b71209e74b54d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Assumptions" sheetId="6" r:id="Rfd7ae984f4844dc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Change Log" sheetId="7" r:id="R131edd1bd6ad40be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Calendar" sheetId="8" r:id="R11f6dba4dcba46ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fast Track Plan" sheetId="9" r:id="Re1c71349dfb84326"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Strategy" sheetId="10" r:id="Rcf8050671aa44fb8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1418,14 +1418,14 @@
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF8EADC4"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF8EADC4"/>
         </x:patternFill>
       </x:fill>
@@ -1762,7 +1762,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ree4c152ca0284402"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R49cc0c2516d54aac"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1792,7 +1792,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb46a72964abf4e9f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc4cd9c90fc24479c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2050,7 +2050,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="237" t="str">
-        <x:v>FDS v3.1.21 · Executive Summary (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.21 · Executive Summary (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="238"/>
       <x:c r="C1" s="238"/>
@@ -2120,7 +2120,7 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="195" t="str">
-        <x:v>v3.1.20 RELEASED / v3.1.21 CANDIDATE</x:v>
+        <x:v>v3.1.21 RELEASED</x:v>
       </x:c>
       <x:c r="D5" s="13" t="str">
         <x:v>D21 decision</x:v>
@@ -2449,10 +2449,10 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>Candidate publication</x:v>
+        <x:v>Publication</x:v>
       </x:c>
       <x:c r="C27" s="67" t="str">
-        <x:v>Independent code review required for mixed PR112.</x:v>
+        <x:v>Content merged; finalization and GitHub Asset verification tracked separately.</x:v>
       </x:c>
       <x:c r="D27" s="198" t="str">
         <x:v>정본 Lead</x:v>
@@ -2491,7 +2491,7 @@
     <x:mergeCell ref="A18:V18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fb943a4ce7f4027"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c4b48de65f84f54"/>
 </x:worksheet>
 </file>
 
@@ -2844,7 +2844,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="237" t="str">
-        <x:v>FDS v3.1.21 · WBS (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.21 · WBS (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="238"/>
       <x:c r="C1" s="238"/>
@@ -2880,7 +2880,7 @@
         </x:is>
       </x:c>
       <x:c r="D2" s="17" t="str">
-        <x:v>v3.1.20 RELEASED / v3.1.21 CANDIDATE</x:v>
+        <x:v>v3.1.21 RELEASED</x:v>
       </x:c>
       <x:c r="E2" s="17" t="inlineStr">
         <x:is>
@@ -7933,7 +7933,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R518b6a7fe24145a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6aa010d7c98e47b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7996,7 +7996,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="237" t="str">
-        <x:v>FDS v3.1.21 · Phase 1 Gantt (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.21 · Phase 1 Gantt (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="238"/>
       <x:c r="C1" s="238"/>
@@ -18153,7 +18153,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="237" t="str">
-        <x:v>FDS v3.1.21 · Phase 2 Gantt (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.21 · Phase 2 Gantt (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="238"/>
       <x:c r="C1" s="238"/>
@@ -25304,7 +25304,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="237" t="str">
-        <x:v>FDS v3.1.21 · Milestones &amp; Decisions (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.21 · Milestones &amp; Decisions (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="238"/>
       <x:c r="C1" s="238"/>
@@ -26709,7 +26709,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="237" t="str">
-        <x:v>FDS v3.1.21 · Risks &amp; Assumptions (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.21 · Risks &amp; Assumptions (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="238"/>
       <x:c r="C1" s="238"/>
@@ -27377,7 +27377,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="237" t="str">
-        <x:v>FDS v3.1.21 · Sources &amp; Change Log (CANDIDATE)</x:v>
+        <x:v>FDS v3.1.21 · Sources &amp; Change Log (RELEASED)</x:v>
       </x:c>
       <x:c r="B1" s="238"/>
       <x:c r="C1" s="238"/>
@@ -27444,7 +27444,7 @@
         <x:v>FDS_Project_Implementation_Baseline_v3.1.21.md</x:v>
       </x:c>
       <x:c r="C4" s="13" t="str">
-        <x:v>v3.1.21 CANDIDATE</x:v>
+        <x:v>v3.1.21 RELEASED</x:v>
       </x:c>
       <x:c r="D4" s="13" t="str">
         <x:v>2026-10-03</x:v>
@@ -28349,10 +28349,8 @@
           <x:t xml:space="preserve">v3.1.20 Phase 2 재계획 (Lead 결정, 2026-09-22)</x:t>
         </x:is>
       </x:c>
-      <x:c r="C34" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">v3.1.20 CANDIDATE</x:t>
-        </x:is>
+      <x:c r="C34" t="str">
+        <x:v>v3.1.20 RELEASED</x:v>
       </x:c>
       <x:c r="D34" t="inlineStr">
         <x:is>
@@ -28455,10 +28453,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
-      <x:c r="A1" s="79" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">FDS v3.1.21 · Team Availability Calendar (CANDIDATE)</x:t>
-        </x:is>
+      <x:c r="A1" s="79" t="str">
+        <x:v>FDS v3.1.21 · Team Availability Calendar (RELEASED)</x:v>
       </x:c>
     </x:row>
     <x:row r="2">

</xml_diff>